<commit_message>
Adicionando a análise do GPT
</commit_message>
<xml_diff>
--- a/GitHub_análise_v1.xlsx
+++ b/GitHub_análise_v1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>Autor</t>
   </si>
@@ -26,88 +26,94 @@
     <t>Daniel Augusto Galleazzo</t>
   </si>
   <si>
-    <t>2025-06-27 23:15:17</t>
-  </si>
-  <si>
-    <t>unahthorized pq o limite de emails ja foi dado</t>
-  </si>
-  <si>
-    <t>2025-06-15 22:45:13</t>
-  </si>
-  <si>
-    <t>começando o java</t>
-  </si>
-  <si>
-    <t>2025-06-11 21:40:09</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Usuário recebe as novas moedas pelo e-mail</t>
-  </si>
-  <si>
-    <t>2025-06-11 13:41:48</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> @Galleazzo me ajudou a pensar na lógica de como melhorar as novas moedas</t>
-  </si>
-  <si>
-    <t>2025-06-11 01:09:16</t>
-  </si>
-  <si>
-    <t>Ver novas moedas</t>
-  </si>
-  <si>
-    <t>2025-06-10 23:36:26</t>
-  </si>
-  <si>
-    <t>Adicionando a terceira opção; pensar melhor parar futuros ajustes</t>
-  </si>
-  <si>
-    <t>2025-06-10 01:52:47</t>
-  </si>
-  <si>
-    <t>Adicionando dois cases</t>
-  </si>
-  <si>
-    <t>2025-06-09 19:22:46</t>
-  </si>
-  <si>
-    <t>Link da imagem</t>
-  </si>
-  <si>
-    <t>2025-06-09 19:01:41</t>
-  </si>
-  <si>
-    <t>Úsuário recebe o horário que as informações foram extraidas</t>
-  </si>
-  <si>
-    <t>2025-06-09 02:24:12</t>
-  </si>
-  <si>
-    <t>Pulando linhas no e-mail cc: @Galleazzo</t>
-  </si>
-  <si>
-    <t>2025-06-09 02:06:43</t>
-  </si>
-  <si>
-    <t>Começando o java</t>
-  </si>
-  <si>
-    <t>2025-06-08 23:18:07</t>
-  </si>
-  <si>
-    <t>Usúario agora pode receber as informações da moeda pelo e-mail</t>
-  </si>
-  <si>
-    <t>2025-06-08 22:02:21</t>
-  </si>
-  <si>
-    <t>Implementando novas coisas</t>
-  </si>
-  <si>
-    <t>2025-06-07 02:26:26</t>
-  </si>
-  <si>
-    <t>PrimeiroCommit</t>
+    <t>2025-06-01 22:16:50</t>
+  </si>
+  <si>
+    <t>Update README.md</t>
+  </si>
+  <si>
+    <t>2025-06-01 22:11:01</t>
+  </si>
+  <si>
+    <t>Add files via upload</t>
+  </si>
+  <si>
+    <t>2025-05-17 01:46:19</t>
+  </si>
+  <si>
+    <t>2025-05-03 15:46:13</t>
+  </si>
+  <si>
+    <t>2025-05-03 14:42:49</t>
+  </si>
+  <si>
+    <t>Remove pasta WindowsFormsTemperatura</t>
+  </si>
+  <si>
+    <t>2025-05-03 05:04:24</t>
+  </si>
+  <si>
+    <t>first commit</t>
+  </si>
+  <si>
+    <t>2025-05-03 04:56:19</t>
+  </si>
+  <si>
+    <t>Adicionando uma interface com WindowsForms</t>
+  </si>
+  <si>
+    <t>2025-05-03 04:31:01</t>
+  </si>
+  <si>
+    <t>Adicionando o WindowsForms</t>
+  </si>
+  <si>
+    <t>2025-05-02 18:01:47</t>
+  </si>
+  <si>
+    <t>Implementação de celsius e fahrenheit</t>
+  </si>
+  <si>
+    <t>2025-05-02 16:12:29</t>
+  </si>
+  <si>
+    <t>Celsius/Fahrenheit</t>
+  </si>
+  <si>
+    <t>2025-05-02 16:09:29</t>
+  </si>
+  <si>
+    <t>Converção de celsius para fahrenheit</t>
+  </si>
+  <si>
+    <t>2025-05-02 15:09:39</t>
+  </si>
+  <si>
+    <t>Removendo</t>
+  </si>
+  <si>
+    <t>2025-05-02 15:08:13</t>
+  </si>
+  <si>
+    <t>Atualização</t>
+  </si>
+  <si>
+    <t>2025-05-01 16:05:52</t>
+  </si>
+  <si>
+    <t>Implementação da interface</t>
+  </si>
+  <si>
+    <t>2025-05-01 03:47:04</t>
+  </si>
+  <si>
+    <t>novas alterações</t>
+  </si>
+  <si>
+    <t>2025-05-01 03:12:45</t>
+  </si>
+  <si>
+    <t>Primeiro commit</t>
   </si>
 </sst>
 </file>
@@ -160,12 +166,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr ">
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24.81122398376465" customWidth="1"/>
     <col min="2" max="2" width="22.434757232666016" customWidth="1"/>
-    <col min="3" max="3" width="76.52838134765625" customWidth="1"/>
+    <col min="3" max="3" width="45.81043243408203" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -209,7 +215,7 @@
         <v>8</v>
       </c>
       <c r="C4" s="0" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -217,10 +223,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C5" s="0" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -228,10 +234,10 @@
         <v>3</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C6" s="0" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
@@ -239,10 +245,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -250,10 +256,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -261,10 +267,10 @@
         <v>3</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
@@ -272,10 +278,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
@@ -283,10 +289,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12">
@@ -294,10 +300,10 @@
         <v>3</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
@@ -305,10 +311,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C13" s="0" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -316,10 +322,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
@@ -327,10 +333,32 @@
         <v>3</v>
       </c>
       <c r="B15" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C16" s="0" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>